<commit_message>
docs: add webhook processing pipeline guide (demo)
- Stripe-quality how-to with HMAC verification (Python + JS)
- Content tabs (Cloud / Self-hosted), Mermaid diagram, admonitions
- Interactive 13-component architecture diagram (5 layers)
- All values from _variables.yml, zero hardcoded values
- Passed 7 linters and 22 SEO/GEO rules on first attempt

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -41,7 +41,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,12 @@
         <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,13 +85,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-04T17:35:50.612234</t>
+          <t>2026-03-07T14:51:27.328474</t>
         </is>
       </c>
     </row>
@@ -504,7 +511,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -516,7 +523,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -528,7 +535,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -540,7 +547,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -552,7 +559,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'code': 10}</t>
+          <t>{'code': 12}</t>
         </is>
       </c>
     </row>
@@ -564,7 +571,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'how-to': 7, 'reference': 3}</t>
+          <t>{'how-to': 8, 'reference': 4}</t>
         </is>
       </c>
     </row>
@@ -576,7 +583,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'authentication': 1, 'database_schema': 1, 'removed_function': 1, 'signature_change': 1, 'new_function': 1, 'webhook': 1, 'public_function': 1, 'config_option': 1, 'env_var': 1, 'error_handling': 1}</t>
+          <t>{'webhook': 1, 'public_function': 1, 'authentication': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'signature_change': 1, 'api_endpoint': 1, 'new_function': 1, 'config_option': 1, 'error_handling': 1, 'env_var': 1}</t>
         </is>
       </c>
     </row>
@@ -591,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -649,12 +656,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-0008</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Authentication: authentication: Auth</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -664,7 +671,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>authentication</t>
+          <t>webhook</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -678,23 +685,23 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>240</v>
+        <v>1239</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in FULL_IMPLEMENTATION_START_HERE.md. Include security considerations.</t>
+          <t>Update webhook documentation for changes in docs/how-to/configure-webhook-trigger.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0503</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -704,12 +711,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>database_schema</t>
+          <t>public_function</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -718,23 +725,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>19</v>
+        <v>846</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in PILOT_VS_FULL_IMPLEMENTATION.md. Update data model documentation.</t>
+          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0100</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: pipeline</t>
+          <t>Authentication: authentication: Auth</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -744,7 +751,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>removed_function</t>
+          <t>authentication</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -758,223 +765,223 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>19</v>
+        <v>756</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function pipeline was removed. Update documentation and add migration guide.</t>
+          <t>Update authentication documentation for changes in docs/.claude/settings.local.json. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0632</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>Database Schema: database_schema: migration</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>database_schema</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Document database schema change in .claude/commands/generate-docs.md. Update data model documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CODE-0622</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>breaking_change</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>URGENT: Document breaking change in .claude/commands/generate-docs.md. Update migration guide with before/after examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CODE-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Removed Function: Function removed: HMAC</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>removed_function</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>BREAKING: Function HMAC was removed. Update documentation and add migration guide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CODE-1138</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>signature_change</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>how-to</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"Found {result['nbHits']} results for 'webhook'") → New: (f"Found {nb_hits} results for 'webhook'"). Update documentation and examples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>CODE-0015</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>New Function: New function: print</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>new_function</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>how-to</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>218</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Document new function: print. Include parameters, return value, and usage example.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>CODE-0001</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Webhook: webhook: webhook</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>webhook</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>how-to</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>170</v>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Update webhook documentation for changes in FULL_IMPLEMENTATION_START_HERE.md. Include payload examples and event types.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>CODE-0141</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Public Function: public_function: seo_validate_file</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>public_function</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"✅ Created {doc_type} document: {output_path}") → New: (f"Created {doc_type} document: {output_path}"). Update documentation and examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CODE-1350</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Api Endpoint: api_endpoint: /webhooks/stripe</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>api_endpoint</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>139</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Consider documenting public API: seo_validate_file. Include parameters, return value, and example usage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>CODE-0008</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Config Option: config_option: local</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>config_option</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Document configuration option: local. Include allowed values and when to use.</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Document API endpoint: /webhooks/stripe. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0189</t>
+          <t>CODE-0473</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Env Var: env_var: ALGOLIA_INDEX_NAME</t>
+          <t>New Function: New function: showInfo</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -984,12 +991,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>env_var</t>
+          <t>new_function</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -998,51 +1005,131 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>4</v>
+        <v>869</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Add environment variable ALGOLIA_INDEX_NAME to configuration reference. Include default value, description, and examples.</t>
+          <t>Document new function: showInfo. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0497</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
+          <t>Config Option: config_option: local</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>config_option</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Document configuration option: local. Include allowed values and when to use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>CODE-1130</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
           <t>Error Handling: error_handling: FileNotFoundError</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>error_handling</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>how-to</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G12" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Document new error type: FileNotFoundError. Include cause, solution, and error code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>CODE-1879</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Env Var: env_var: DATABASE_URL</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>env_var</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Add environment variable DATABASE_URL to configuration reference. Include default value, description, and examples.</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1115,12 +1202,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-0008</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Authentication: authentication: Auth</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1130,7 +1217,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>authentication</t>
+          <t>webhook</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -1144,23 +1231,23 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>240</v>
+        <v>1239</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in FULL_IMPLEMENTATION_START_HERE.md. Include security considerations.</t>
+          <t>Update webhook documentation for changes in docs/how-to/configure-webhook-trigger.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0503</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1170,12 +1257,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>database_schema</t>
+          <t>public_function</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1184,23 +1271,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>19</v>
+        <v>846</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in PILOT_VS_FULL_IMPLEMENTATION.md. Update data model documentation.</t>
+          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0100</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: pipeline</t>
+          <t>Authentication: authentication: Auth</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1210,7 +1297,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>removed_function</t>
+          <t>authentication</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1224,51 +1311,211 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>19</v>
+        <v>756</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function pipeline was removed. Update documentation and add migration guide.</t>
+          <t>Update authentication documentation for changes in docs/.claude/settings.local.json. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0632</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>Database Schema: database_schema: migration</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>database_schema</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Document database schema change in .claude/commands/generate-docs.md. Update data model documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CODE-0622</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>breaking_change</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>URGENT: Document breaking change in .claude/commands/generate-docs.md. Update migration guide with before/after examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CODE-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Removed Function: Function removed: HMAC</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>removed_function</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>BREAKING: Function HMAC was removed. Update documentation and add migration guide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CODE-1138</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>signature_change</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>how-to</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"Found {result['nbHits']} results for 'webhook'") → New: (f"Found {nb_hits} results for 'webhook'"). Update documentation and examples.</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"✅ Created {doc_type} document: {output_path}") → New: (f"Created {doc_type} document: {output_path}"). Update documentation and examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CODE-1350</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Api Endpoint: api_endpoint: /webhooks/stripe</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>api_endpoint</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Document API endpoint: /webhooks/stripe. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
@@ -1294,19 +1541,19 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>(10 gaps)</t>
+          <t>(12 gaps)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-0008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Authentication: authentication: Auth</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1318,12 +1565,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0503</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1335,12 +1582,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0100</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: pipeline</t>
+          <t>Authentication: authentication: Auth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1352,12 +1599,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0632</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: print</t>
+          <t>Database Schema: database_schema: migration</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1369,80 +1616,80 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0015</t>
+          <t>CODE-0622</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New Function: New function: print</t>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Removed Function: Function removed: HMAC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-0141</t>
+          <t>CODE-1138</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Public Function: public_function: seo_validate_file</t>
+          <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-0008</t>
+          <t>CODE-1350</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Config Option: config_option: local</t>
+          <t>Api Endpoint: api_endpoint: /webhooks/stripe</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0189</t>
+          <t>CODE-0473</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Env Var: env_var: ALGOLIA_INDEX_NAME</t>
+          <t>New Function: New function: showInfo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1454,12 +1701,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0497</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: FileNotFoundError</t>
+          <t>Config Option: config_option: local</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
Finalize client onboarding, automation, and docs updates
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-07T19:41:56.166063</t>
+          <t>2026-03-11T11:24:07.191737</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'webhook': 1, 'authentication': 1, 'public_function': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'api_endpoint': 1, 'signature_change': 1, 'new_function': 1, 'config_option': 1, 'error_handling': 1, 'env_var': 1}</t>
+          <t>{'webhook': 1, 'authentication': 1, 'public_function': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'api_endpoint': 1, 'signature_change': 1, 'new_function': 1, 'error_handling': 1, 'config_option': 1, 'env_var': 1}</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -678,18 +678,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1805</v>
+        <v>2663</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in .claude/skills/demo/SKILL.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0019</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -718,23 +718,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>721</v>
+        <v>1447</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0031</t>
+          <t>CODE-0083</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: now_iso</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -758,23 +758,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>709</v>
+        <v>822</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: now_iso. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0818</t>
+          <t>CODE-0124</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Database Schema: database_schema: CREATE TABLE</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -798,18 +798,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in reports/doc_gaps_report.csv. Update data model documentation.</t>
+          <t>Document database schema change in sandbox/prodlike_api/app/main.py. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0788</t>
+          <t>CODE-0330</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -838,23 +838,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
+          <t>URGENT: Document breaking change in reports/consolidated_report.json. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0224</t>
+          <t>CODE-1209</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: Say</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -878,23 +878,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function Say was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0096</t>
+          <t>CODE-2097</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /webhooks</t>
+          <t>Api Endpoint: api_endpoint: /healthz</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -918,18 +918,18 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /webhooks. Include request/response examples, parameters, authentication requirements.</t>
+          <t>Document API endpoint: /healthz. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-2154</t>
+          <t>CODE-4596</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -969,12 +969,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0045</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: if</t>
+          <t>New Function: New function: startup</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -998,23 +998,23 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>669</v>
+        <v>845</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: if. Include parameters, return value, and usage example.</t>
+          <t>Document new function: startup. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0264</t>
+          <t>CODE-0278</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Config Option: config_option: local</t>
+          <t>Error Handling: error_handling: RuntimeError</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1024,12 +1024,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>config_option</t>
+          <t>error_handling</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1038,23 +1038,23 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Document configuration option: local. Include allowed values and when to use.</t>
+          <t>Document new error type: RuntimeError. Include cause, solution, and error code.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0352</t>
+          <t>CODE-0329</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: 401</t>
+          <t>Config Option: config_option: local</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1064,12 +1064,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>error_handling</t>
+          <t>config_option</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1078,23 +1078,23 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Document new error type: 401. Include cause, solution, and error code.</t>
+          <t>Document configuration option: local. Include allowed values and when to use.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CODE-0303</t>
+          <t>CODE-2042</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Env Var: env_var: WEBHOOK_SECRET</t>
+          <t>Env Var: env_var: ASK_AI_API_KEY</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1118,11 +1118,11 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Add environment variable WEBHOOK_SECRET to configuration reference. Include default value, description, and examples.</t>
+          <t>Add environment variable ASK_AI_API_KEY to configuration reference. Include default value, description, and examples.</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -1224,18 +1224,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1805</v>
+        <v>2663</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in .claude/skills/demo/SKILL.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0019</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -1264,23 +1264,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>721</v>
+        <v>1447</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0031</t>
+          <t>CODE-0083</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: now_iso</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1304,23 +1304,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>709</v>
+        <v>822</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: now_iso. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0818</t>
+          <t>CODE-0124</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Database Schema: database_schema: CREATE TABLE</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1344,18 +1344,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in reports/doc_gaps_report.csv. Update data model documentation.</t>
+          <t>Document database schema change in sandbox/prodlike_api/app/main.py. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0788</t>
+          <t>CODE-0330</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1384,23 +1384,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
+          <t>URGENT: Document breaking change in reports/consolidated_report.json. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0224</t>
+          <t>CODE-1209</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: Say</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1424,23 +1424,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function Say was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0096</t>
+          <t>CODE-2097</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /webhooks</t>
+          <t>Api Endpoint: api_endpoint: /healthz</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1464,18 +1464,18 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /webhooks. Include request/response examples, parameters, authentication requirements.</t>
+          <t>Document API endpoint: /healthz. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-2154</t>
+          <t>CODE-4596</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1558,7 +1558,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CODE-0019</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0031</t>
+          <t>CODE-0083</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: now_iso</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1592,12 +1592,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0818</t>
+          <t>CODE-0124</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Database Schema: database_schema: CREATE TABLE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1609,7 +1609,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0788</t>
+          <t>CODE-0330</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0224</t>
+          <t>CODE-1209</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: Say</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1643,12 +1643,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-0096</t>
+          <t>CODE-2097</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /webhooks</t>
+          <t>Api Endpoint: api_endpoint: /healthz</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1660,7 +1660,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-2154</t>
+          <t>CODE-4596</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0045</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: if</t>
+          <t>New Function: New function: startup</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,12 +1694,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0264</t>
+          <t>CODE-0278</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Config Option: config_option: local</t>
+          <t>Error Handling: error_handling: RuntimeError</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
Fix demo guardrails and normalize list handling
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-11T11:24:07.191737</t>
+          <t>2026-03-11T15:28:41.745644</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0002</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -678,18 +678,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2663</v>
+        <v>3064</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in .claude/skills/demo/SKILL.md. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0005</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -718,23 +718,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1447</v>
+        <v>1813</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
+          <t>Update authentication documentation for changes in mkdocs.yml. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0083</t>
+          <t>CODE-0075</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: now_iso</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -758,23 +758,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>822</v>
+        <v>965</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: now_iso. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0124</t>
+          <t>CODE-0147</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: CREATE TABLE</t>
+          <t>Database Schema: database_schema: migration</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -798,23 +798,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in sandbox/prodlike_api/app/main.py. Update data model documentation.</t>
+          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0330</t>
+          <t>CODE-0684</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Breaking Change: breaking_change: </t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-1209</t>
+          <t>CODE-0006</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -889,12 +889,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-2097</t>
+          <t>CODE-1078</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /healthz</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -918,23 +918,23 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /healthz. Include request/response examples, parameters, authentication requirements.</t>
+          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-4596</t>
+          <t>CODE-0859</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: print</t>
+          <t>Signature Change: Function signature changed: __init__</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -958,23 +958,23 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"✅ Created {doc_type} document: {output_path}") → New: (f"Created {doc_type} document: {output_path}"). Update documentation and examples.</t>
+          <t>UPDATE REQUIRED: Function __init__ signature changed. Old: (self, docs_dir: str = "docs") → New: (self, docs_dir: str = "docs", policy_pack_path: str | None = None). Update documentation and examples.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0045</t>
+          <t>CODE-0056</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: startup</t>
+          <t>New Function: New function: showInfo</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -998,23 +998,23 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>845</v>
+        <v>1006</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: startup. Include parameters, return value, and usage example.</t>
+          <t>Document new function: showInfo. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0278</t>
+          <t>CODE-0849</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: RuntimeError</t>
+          <t>Error Handling: error_handling: ValueError</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1038,18 +1038,18 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Document new error type: RuntimeError. Include cause, solution, and error code.</t>
+          <t>Document new error type: ValueError. Include cause, solution, and error code.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0329</t>
+          <t>CODE-0178</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CODE-2042</t>
+          <t>CODE-3228</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0002</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1224,18 +1224,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2663</v>
+        <v>3064</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in .claude/skills/demo/SKILL.md. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0005</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -1264,23 +1264,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1447</v>
+        <v>1813</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
+          <t>Update authentication documentation for changes in mkdocs.yml. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0083</t>
+          <t>CODE-0075</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: now_iso</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1304,23 +1304,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>822</v>
+        <v>965</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: now_iso. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0124</t>
+          <t>CODE-0147</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: CREATE TABLE</t>
+          <t>Database Schema: database_schema: migration</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1344,23 +1344,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in sandbox/prodlike_api/app/main.py. Update data model documentation.</t>
+          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0330</t>
+          <t>CODE-0684</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Breaking Change: breaking_change: </t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-1209</t>
+          <t>CODE-0006</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -1435,12 +1435,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-2097</t>
+          <t>CODE-1078</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /healthz</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1464,23 +1464,23 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /healthz. Include request/response examples, parameters, authentication requirements.</t>
+          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-4596</t>
+          <t>CODE-0859</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: print</t>
+          <t>Signature Change: Function signature changed: __init__</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1504,11 +1504,11 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function print signature changed. Old: (f"✅ Created {doc_type} document: {output_path}") → New: (f"Created {doc_type} document: {output_path}"). Update documentation and examples.</t>
+          <t>UPDATE REQUIRED: Function __init__ signature changed. Old: (self, docs_dir: str = "docs") → New: (self, docs_dir: str = "docs", policy_pack_path: str | None = None). Update documentation and examples.</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0002</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1558,7 +1558,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0005</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0083</t>
+          <t>CODE-0075</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Public Function: public_function: now_iso</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1592,12 +1592,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0124</t>
+          <t>CODE-0147</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: CREATE TABLE</t>
+          <t>Database Schema: database_schema: migration</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1609,12 +1609,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0330</t>
+          <t>CODE-0684</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Breaking Change: breaking_change: </t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-1209</t>
+          <t>CODE-0006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1643,12 +1643,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-2097</t>
+          <t>CODE-1078</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /healthz</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1660,12 +1660,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-4596</t>
+          <t>CODE-0859</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: print</t>
+          <t>Signature Change: Function signature changed: __init__</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0045</t>
+          <t>CODE-0056</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: startup</t>
+          <t>New Function: New function: showInfo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,12 +1694,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0278</t>
+          <t>CODE-0849</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: RuntimeError</t>
+          <t>Error Handling: error_handling: ValueError</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
fix: remediate CI/deploy failure in demo loop
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-11T15:28:41.745644</t>
+          <t>2026-03-11T15:53:23.662950</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: Webhook</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -678,18 +678,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3064</v>
+        <v>3230</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in .claude/commands/demo.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -718,18 +718,18 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1813</v>
+        <v>1900</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in mkdocs.yml. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0075</t>
+          <t>CODE-0394</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0147</t>
+          <t>CODE-0036</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -798,23 +798,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>205</v>
+        <v>232</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
+          <t>Document database schema change in reports/batch_tasks.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0684</t>
+          <t>CODE-0009</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -838,23 +838,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/consolidated_report.json. Update migration guide with before/after examples.</t>
+          <t>URGENT: Document breaking change in reports/batch_tasks.json. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0006</t>
+          <t>CODE-0193</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: showInfo</t>
+          <t>Removed Function: Function removed: selectPack</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -878,18 +878,18 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function selectPack was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-1078</t>
+          <t>CODE-1397</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -929,7 +929,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-0859</t>
+          <t>CODE-1178</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -969,12 +969,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0056</t>
+          <t>CODE-0375</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: showInfo</t>
+          <t>New Function: New function: if</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1002,14 +1002,14 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: showInfo. Include parameters, return value, and usage example.</t>
+          <t>Document new function: if. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0849</t>
+          <t>CODE-1168</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1049,7 +1049,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0178</t>
+          <t>CODE-0064</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CODE-3228</t>
+          <t>CODE-3547</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: Webhook</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1224,18 +1224,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3064</v>
+        <v>3230</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in .claude/commands/demo.md. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -1264,18 +1264,18 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1813</v>
+        <v>1900</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in mkdocs.yml. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0075</t>
+          <t>CODE-0394</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0147</t>
+          <t>CODE-0036</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1344,23 +1344,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>205</v>
+        <v>232</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
+          <t>Document database schema change in reports/batch_tasks.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0684</t>
+          <t>CODE-0009</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1384,23 +1384,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/consolidated_report.json. Update migration guide with before/after examples.</t>
+          <t>URGENT: Document breaking change in reports/batch_tasks.json. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0006</t>
+          <t>CODE-0193</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: showInfo</t>
+          <t>Removed Function: Function removed: selectPack</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1424,18 +1424,18 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function selectPack was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-1078</t>
+          <t>CODE-1397</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-0859</t>
+          <t>CODE-1178</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Webhook: webhook: Webhook</t>
+          <t>Webhook: webhook: webhook</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1558,7 +1558,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CODE-0005</t>
+          <t>CODE-0004</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0075</t>
+          <t>CODE-0394</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0147</t>
+          <t>CODE-0036</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1609,12 +1609,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0684</t>
+          <t>CODE-0009</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t xml:space="preserve">Breaking Change: breaking_change: </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0006</t>
+          <t>CODE-0193</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: showInfo</t>
+          <t>Removed Function: Function removed: selectPack</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1643,7 +1643,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-1078</t>
+          <t>CODE-1397</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1660,7 +1660,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-0859</t>
+          <t>CODE-1178</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0056</t>
+          <t>CODE-0375</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: showInfo</t>
+          <t>New Function: New function: if</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0849</t>
+          <t>CODE-1168</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">

</xml_diff>

<commit_message>
chore: update demo artifacts and articulate glossary sync stage
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-11T18:34:07.552810</t>
+          <t>2026-03-12T12:14:23.030117</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'webhook': 1, 'authentication': 1, 'public_function': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'api_endpoint': 1, 'signature_change': 1, 'new_function': 1, 'error_handling': 1, 'config_option': 1, 'env_var': 1}</t>
+          <t>{'webhook': 1, 'authentication': 1, 'public_function': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'signature_change': 1, 'api_endpoint': 1, 'new_function': 1, 'error_handling': 1, 'config_option': 1, 'env_var': 1}</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0052</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: retrieval_evals_report.json</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -678,18 +678,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4074</v>
+        <v>4482</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in scripts/consolidate_reports.py. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0016</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -718,23 +718,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2028</v>
+        <v>2148</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0230</t>
+          <t>CODE-0064</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: build_graph</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -758,18 +758,18 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>968</v>
+        <v>386</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: build_graph. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0539</t>
+          <t>CODE-0127</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -798,18 +798,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>251</v>
+        <v>208</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in reports/doc_gaps_report.csv. Update data model documentation.</t>
+          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0515</t>
+          <t>CODE-0925</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -849,12 +849,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0188</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: if</t>
+          <t>Removed Function: Function removed: return</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -878,23 +878,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function if was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function return was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-2436</t>
+          <t>CODE-0746</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
+          <t>Signature Change: Function signature changed: _run_python</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -904,12 +904,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>api_endpoint</t>
+          <t>signature_change</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -922,19 +922,19 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
+          <t>UPDATE REQUIRED: Function _run_python signature changed. Old: (content: str, timeout: int) → New: (content: str, timeout: int, execute: bool). Update documentation and examples.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-2217</t>
+          <t>CODE-3978</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: __init__</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -944,12 +944,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>signature_change</t>
+          <t>api_endpoint</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -958,23 +958,23 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function __init__ signature changed. Old: (self, docs_dir: str = "docs") → New: (self, docs_dir: str = "docs", policy_pack_path: str | None = None). Update documentation and examples.</t>
+          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0205</t>
+          <t>CODE-0049</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: if</t>
+          <t>New Function: New function: _process_retrieval_evals</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -998,18 +998,18 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>1022</v>
+        <v>570</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: if. Include parameters, return value, and usage example.</t>
+          <t>Document new function: _process_retrieval_evals. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-2207</t>
+          <t>CODE-0101</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
@@ -1049,12 +1049,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0566</t>
+          <t>CODE-0034</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Config Option: config_option: local</t>
+          <t>Config Option: config_option: billing_mode</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1078,18 +1078,18 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Document configuration option: local. Include allowed values and when to use.</t>
+          <t>Document configuration option: billing_mode. Include allowed values and when to use.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CODE-4586</t>
+          <t>CODE-6128</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
@@ -1195,12 +1195,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0052</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: retrieval_evals_report.json</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1224,18 +1224,18 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4074</v>
+        <v>4482</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in scripts/consolidate_reports.py. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CODE-0016</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -1264,23 +1264,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2028</v>
+        <v>2148</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in docs/diagrams/demo-webhook-pipeline.html. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0230</t>
+          <t>CODE-0064</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: build_graph</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1304,18 +1304,18 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>968</v>
+        <v>386</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: build_graph. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0539</t>
+          <t>CODE-0127</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1344,18 +1344,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>251</v>
+        <v>208</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in reports/doc_gaps_report.csv. Update data model documentation.</t>
+          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0515</t>
+          <t>CODE-0925</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -1395,12 +1395,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0188</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: if</t>
+          <t>Removed Function: Function removed: return</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1424,23 +1424,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function if was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function return was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-2436</t>
+          <t>CODE-0746</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
+          <t>Signature Change: Function signature changed: _run_python</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1450,12 +1450,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>api_endpoint</t>
+          <t>signature_change</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1468,19 +1468,19 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
+          <t>UPDATE REQUIRED: Function _run_python signature changed. Old: (content: str, timeout: int) → New: (content: str, timeout: int, execute: bool). Update documentation and examples.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-2217</t>
+          <t>CODE-3978</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: __init__</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>signature_change</t>
+          <t>api_endpoint</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1504,11 +1504,11 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function __init__ signature changed. Old: (self, docs_dir: str = "docs") → New: (self, docs_dir: str = "docs", policy_pack_path: str | None = None). Update documentation and examples.</t>
+          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0004</t>
+          <t>CODE-0052</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Webhook: webhook: webhook</t>
+          <t>Webhook: webhook: retrieval_evals_report.json</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1558,7 +1558,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CODE-0016</t>
+          <t>CODE-0001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0230</t>
+          <t>CODE-0064</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Public Function: public_function: verify_webhook_signature</t>
+          <t>Public Function: public_function: build_graph</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0539</t>
+          <t>CODE-0127</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1609,7 +1609,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0515</t>
+          <t>CODE-0925</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0001</t>
+          <t>CODE-0188</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: if</t>
+          <t>Removed Function: Function removed: return</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1643,12 +1643,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-2436</t>
+          <t>CODE-0746</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
+          <t>Signature Change: Function signature changed: _run_python</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1660,12 +1660,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-2217</t>
+          <t>CODE-3978</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: __init__</t>
+          <t>Api Endpoint: api_endpoint: /tasks</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0205</t>
+          <t>CODE-0049</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: if</t>
+          <t>New Function: New function: _process_retrieval_evals</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-2207</t>
+          <t>CODE-0101</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">

</xml_diff>

<commit_message>
docs: add US commercial one-pager and update generated docs artifacts
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-12T12:14:23.030117</t>
+          <t>2026-03-13T16:02:56.954024</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0052</t>
+          <t>CODE-0029</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: retrieval_evals_report.json</t>
+          <t>Webhook: webhook: pr_docs_contract.json</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4482</v>
+        <v>4889</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
@@ -718,23 +718,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2148</v>
+        <v>2407</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .gitignore. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0064</t>
+          <t>CODE-0037</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: build_graph</t>
+          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -758,18 +758,18 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>386</v>
+        <v>438</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: build_graph. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: test_emits_only_new_or_changed_items. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0127</t>
+          <t>CODE-0003</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -798,18 +798,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>208</v>
+        <v>227</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
+          <t>Document database schema change in API_FIRST_PLAYBOOK.md. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0925</t>
+          <t>CODE-0757</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -849,12 +849,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0134</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: return</t>
+          <t>Removed Function: Function removed: print</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -878,23 +878,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function return was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function print was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0746</t>
+          <t>CODE-0022</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: _run_python</t>
+          <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -918,18 +918,18 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function _run_python signature changed. Old: (content: str, timeout: int) → New: (content: str, timeout: int, execute: bool). Update documentation and examples.</t>
+          <t>UPDATE REQUIRED: Function print signature changed. Old: ("Blocking PR: public interface changed but docs were not updated.") → New: ("Docs contract drift found (report-only mode). Update documentation and examples.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-3978</t>
+          <t>CODE-4848</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -969,12 +969,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0049</t>
+          <t>CODE-0024</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: _process_retrieval_evals</t>
+          <t>New Function: New function: _dod_duplicate_exists</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -998,23 +998,23 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>570</v>
+        <v>649</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: _process_retrieval_evals. Include parameters, return value, and usage example.</t>
+          <t>Document new function: _dod_duplicate_exists. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0101</t>
+          <t>CODE-0314</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: ValueError</t>
+          <t>Error Handling: error_handling: RuntimeError</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1038,18 +1038,18 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Document new error type: ValueError. Include cause, solution, and error code.</t>
+          <t>Document new error type: RuntimeError. Include cause, solution, and error code.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0034</t>
+          <t>CODE-0904</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CODE-6128</t>
+          <t>CODE-6998</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0052</t>
+          <t>CODE-0029</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: retrieval_evals_report.json</t>
+          <t>Webhook: webhook: pr_docs_contract.json</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4482</v>
+        <v>4889</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
@@ -1264,23 +1264,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2148</v>
+        <v>2407</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .claude/commands/api-first-demo.md. Include security considerations.</t>
+          <t>Update authentication documentation for changes in .gitignore. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0064</t>
+          <t>CODE-0037</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: build_graph</t>
+          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1304,18 +1304,18 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>386</v>
+        <v>438</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: build_graph. Include parameters, return value, and example usage.</t>
+          <t>Consider documenting public API: test_emits_only_new_or_changed_items. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0127</t>
+          <t>CODE-0003</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1344,18 +1344,18 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>208</v>
+        <v>227</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in seo-report-algolia.json. Update data model documentation.</t>
+          <t>Document database schema change in API_FIRST_PLAYBOOK.md. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0925</t>
+          <t>CODE-0757</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -1395,12 +1395,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0134</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: return</t>
+          <t>Removed Function: Function removed: print</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1424,23 +1424,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function return was removed. Update documentation and add migration guide.</t>
+          <t>BREAKING: Function print was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0746</t>
+          <t>CODE-0022</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: _run_python</t>
+          <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1464,18 +1464,18 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>UPDATE REQUIRED: Function _run_python signature changed. Old: (content: str, timeout: int) → New: (content: str, timeout: int, execute: bool). Update documentation and examples.</t>
+          <t>UPDATE REQUIRED: Function print signature changed. Old: ("Blocking PR: public interface changed but docs were not updated.") → New: ("Docs contract drift found (report-only mode). Update documentation and examples.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CODE-3978</t>
+          <t>CODE-4848</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1541,12 +1541,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0052</t>
+          <t>CODE-0029</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Webhook: webhook: retrieval_evals_report.json</t>
+          <t>Webhook: webhook: pr_docs_contract.json</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0064</t>
+          <t>CODE-0037</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Public Function: public_function: build_graph</t>
+          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0127</t>
+          <t>CODE-0003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1609,7 +1609,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0925</t>
+          <t>CODE-0757</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0188</t>
+          <t>CODE-0134</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: return</t>
+          <t>Removed Function: Function removed: print</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1643,12 +1643,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-0746</t>
+          <t>CODE-0022</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Signature Change: Function signature changed: _run_python</t>
+          <t>Signature Change: Function signature changed: print</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1660,7 +1660,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-3978</t>
+          <t>CODE-4848</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0049</t>
+          <t>CODE-0024</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: _process_retrieval_evals</t>
+          <t>New Function: New function: _dod_duplicate_exists</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,12 +1694,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0101</t>
+          <t>CODE-0314</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: ValueError</t>
+          <t>Error Handling: error_handling: RuntimeError</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
chore: add pending changes from recent sessions
Includes client bundle tooling, confluence migration scripts,
knowledge modules, operator questionnaire, pricing/upsell playbooks,
pilot-evidence preset, finalize docs gate, audit scorecard reports,
and various operations docs and config updates.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/doc_gaps_report.xlsx
+++ b/reports/doc_gaps_report.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-13T16:02:56.954024</t>
+          <t>2026-03-17T15:41:33.465903</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'code': 12}</t>
+          <t>{'code': 11}</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'how-to': 8, 'reference': 4}</t>
+          <t>{'how-to': 8, 'reference': 3}</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'webhook': 1, 'authentication': 1, 'public_function': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'signature_change': 1, 'api_endpoint': 1, 'new_function': 1, 'error_handling': 1, 'config_option': 1, 'env_var': 1}</t>
+          <t>{'webhook': 1, 'authentication': 1, 'database_schema': 1, 'breaking_change': 1, 'removed_function': 1, 'api_endpoint': 1, 'signature_change': 1, 'new_function': 1, 'public_function': 1, 'error_handling': 1, 'config_option': 1}</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -649,12 +649,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0029</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: pr_docs_contract.json</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -678,11 +678,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4889</v>
+        <v>3832</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in scripts/consolidate_reports.py. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
@@ -718,23 +718,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2407</v>
+        <v>1915</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .gitignore. Include security considerations.</t>
+          <t>Update authentication documentation for changes in docs/reference/taskstream-api-playground.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0037</t>
+          <t>CODE-0976</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
+          <t>Database Schema: database_schema: schema(</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>public_function</t>
+          <t>database_schema</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -758,23 +758,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>438</v>
+        <v>213</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: test_emits_only_new_or_changed_items. Include parameters, return value, and example usage.</t>
+          <t>Document database schema change in scripts/generate_api_test_assets.py. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-1131</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>database_schema</t>
+          <t>breaking_change</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -798,23 +798,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>227</v>
+        <v>100</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in API_FIRST_PLAYBOOK.md. Update data model documentation.</t>
+          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0757</t>
+          <t>CODE-0237</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>breaking_change</t>
+          <t>removed_function</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -838,23 +838,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
+          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0134</t>
+          <t>CODE-0268</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: print</t>
+          <t>Api Endpoint: api_endpoint: /webhooks</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>removed_function</t>
+          <t>api_endpoint</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -878,18 +878,18 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function print was removed. Update documentation and add migration guide.</t>
+          <t>Document API endpoint: /webhooks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0022</t>
+          <t>CODE-2304</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -927,54 +927,54 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CODE-4848</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>api_endpoint</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>CODE-0343</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>New Function: New function: _not_implemented</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>new_function</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>how-to</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>587</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Document new function: _not_implemented. Include parameters, return value, and usage example.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CODE-0024</t>
+          <t>CODE-0634</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>New Function: New function: _dod_duplicate_exists</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>new_function</t>
+          <t>public_function</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -998,23 +998,23 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>649</v>
+        <v>349</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Document new function: _dod_duplicate_exists. Include parameters, return value, and usage example.</t>
+          <t>Consider documenting public API: verify_webhook_signature. Include parameters, return value, and example usage.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CODE-0314</t>
+          <t>CODE-0341</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: RuntimeError</t>
+          <t>Error Handling: error_handling: 401</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1038,23 +1038,23 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Document new error type: RuntimeError. Include cause, solution, and error code.</t>
+          <t>Document new error type: 401. Include cause, solution, and error code.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CODE-0904</t>
+          <t>CODE-1256</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Config Option: config_option: billing_mode</t>
+          <t>Config Option: config_option: local</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1078,51 +1078,11 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Document configuration option: billing_mode. Include allowed values and when to use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>CODE-6998</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Env Var: env_var: ASK_AI_API_KEY</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>env_var</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Add environment variable ASK_AI_API_KEY to configuration reference. Include default value, description, and examples.</t>
+          <t>Document configuration option: local. Include allowed values and when to use.</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1195,12 +1155,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CODE-0029</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Webhook: webhook: pr_docs_contract.json</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1224,11 +1184,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4889</v>
+        <v>3832</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Update webhook documentation for changes in scripts/consolidate_reports.py. Include payload examples and event types.</t>
+          <t>Update webhook documentation for changes in mkdocs.yml. Include payload examples and event types.</t>
         </is>
       </c>
     </row>
@@ -1264,23 +1224,23 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2407</v>
+        <v>1915</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Update authentication documentation for changes in .gitignore. Include security considerations.</t>
+          <t>Update authentication documentation for changes in docs/reference/taskstream-api-playground.md. Include security considerations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CODE-0037</t>
+          <t>CODE-0976</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
+          <t>Database Schema: database_schema: schema(</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1290,12 +1250,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>public_function</t>
+          <t>database_schema</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>how-to</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1304,23 +1264,23 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>438</v>
+        <v>213</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Consider documenting public API: test_emits_only_new_or_changed_items. Include parameters, return value, and example usage.</t>
+          <t>Document database schema change in scripts/generate_api_test_assets.py. Update data model documentation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-1131</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1330,7 +1290,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>database_schema</t>
+          <t>breaking_change</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1344,23 +1304,23 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>227</v>
+        <v>100</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Document database schema change in API_FIRST_PLAYBOOK.md. Update data model documentation.</t>
+          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CODE-0757</t>
+          <t>CODE-0237</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1370,7 +1330,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>breaking_change</t>
+          <t>removed_function</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1384,23 +1344,23 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>URGENT: Document breaking change in reports/doc_gaps_report.csv. Update migration guide with before/after examples.</t>
+          <t>BREAKING: Function showInfo was removed. Update documentation and add migration guide.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CODE-0134</t>
+          <t>CODE-0268</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: print</t>
+          <t>Api Endpoint: api_endpoint: /webhooks</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1410,12 +1370,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>removed_function</t>
+          <t>api_endpoint</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>how-to</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1424,18 +1384,18 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>BREAKING: Function print was removed. Update documentation and add migration guide.</t>
+          <t>Document API endpoint: /webhooks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CODE-0022</t>
+          <t>CODE-2304</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1469,46 +1429,6 @@
       <c r="H8" s="4" t="inlineStr">
         <is>
           <t>UPDATE REQUIRED: Function print signature changed. Old: ("Blocking PR: public interface changed but docs were not updated.") → New: ("Docs contract drift found (report-only mode). Update documentation and examples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CODE-4848</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>api_endpoint</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Document API endpoint: /tasks. Include request/response examples, parameters, authentication requirements.</t>
         </is>
       </c>
     </row>
@@ -1534,19 +1454,19 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>(12 gaps)</t>
+          <t>(11 gaps)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CODE-0029</t>
+          <t>CODE-0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Webhook: webhook: pr_docs_contract.json</t>
+          <t>Webhook: webhook: Webhook</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1575,12 +1495,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CODE-0037</t>
+          <t>CODE-0976</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Public Function: public_function: test_emits_only_new_or_changed...</t>
+          <t>Database Schema: database_schema: schema(</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1592,12 +1512,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CODE-0003</t>
+          <t>CODE-1131</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Database Schema: database_schema: migration</t>
+          <t>Breaking Change: breaking_change:  Change</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1609,12 +1529,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CODE-0757</t>
+          <t>CODE-0237</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Breaking Change: breaking_change:  Change</t>
+          <t>Removed Function: Function removed: showInfo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1626,12 +1546,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CODE-0134</t>
+          <t>CODE-0268</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Removed Function: Function removed: print</t>
+          <t>Api Endpoint: api_endpoint: /webhooks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1643,7 +1563,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CODE-0022</t>
+          <t>CODE-2304</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1660,29 +1580,29 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CODE-4848</t>
+          <t>CODE-0343</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Api Endpoint: api_endpoint: /tasks</t>
+          <t>New Function: New function: _not_implemented</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CODE-0024</t>
+          <t>CODE-0634</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Function: New function: _dod_duplicate_exists</t>
+          <t>Public Function: public_function: verify_webhook_signature</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1694,12 +1614,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CODE-0314</t>
+          <t>CODE-0341</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error Handling: error_handling: RuntimeError</t>
+          <t>Error Handling: error_handling: 401</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>